<commit_message>
Pull all voter data into the Capital Workbook
Added three voter-data tabs + Summary voter-signal KPIs so the data and
the case live in one file:
- Capital & Special Votes: 16 capital/reserve/bond/governance articles
  (2015-2026) with computed % YES and pass/fail vs threshold — shows
  reserves/credits clear easily while facility bonds win majorities but
  die at the 3/5 wall
- Budget Votes: operating-budget margins by meeting year 2012-2026
  (support ~81% -> 57%), with as-voted % computed
- Board Elections: Select Board races & turnover 2022-2026
- Summary now carries voter-signal KPIs tying the vote history to why the
  reserve+aid financing fits this electorate

Workbook now 9 tabs.

https://claude.ai/code/session_01QjR1e91vo6hzvZdpnVX6Mh
</commit_message>
<xml_diff>
--- a/docs/analyses/swanzey-capital-forecast/Swanzey Capital Workbook.xlsx
+++ b/docs/analyses/swanzey-capital-forecast/Swanzey Capital Workbook.xlsx
@@ -12,7 +12,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reserve Ladder" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10-Year Plan" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bridge Aid Calc" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capital &amp; Special Votes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget Votes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Board Elections" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +30,7 @@
     <numFmt numFmtId="166" formatCode="$#,##0;[Red]-$#,##0"/>
     <numFmt numFmtId="167" formatCode="$0.00"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,6 +69,18 @@
       <b val="1"/>
       <color rgb="001F3A5F"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000F6E56"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00993C1D"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00993C1D"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -102,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -128,6 +143,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -599,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -716,9 +734,57 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>You can't beat a failed 3/5 bond with a better speech — restructure the money. Save via majority-vote reserves; let state aid, water rates, and grants carry ~62%.</t>
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Voter signals (why the financing fits)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Reserves &amp; tax credits — pass rate</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>78–90%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Facility bonds passed (need 3/5)</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>0 of 2 — failed 2024 &amp; 2026 with majorities</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Operating-budget support, 2011 → 2025</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>~81% → 57%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2025 capital activity</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>acquired West Swanzey water; funded SRF study; board 3→5</t>
         </is>
       </c>
     </row>
@@ -1830,6 +1896,1317 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Capital &amp; Special Warrant Votes — the historical pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>% YES computed. Note: reserves &amp; credits clear easily; facility BONDS win majorities but die at the 3/5 wall.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>% YES</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Threshold</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Capital / borrowing</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>578</v>
+      </c>
+      <c r="F5" t="n">
+        <v>294</v>
+      </c>
+      <c r="G5" s="10">
+        <f>E5/(E5+F5)</f>
+        <v/>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>3/5</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Capital reserve deposit</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>272000</v>
+      </c>
+      <c r="E6" t="n">
+        <v>470</v>
+      </c>
+      <c r="F6" t="n">
+        <v>178</v>
+      </c>
+      <c r="G6" s="10">
+        <f>E6/(E6+F6)</f>
+        <v/>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>majority</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Capital reserve deposit</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>590000</v>
+      </c>
+      <c r="E7" t="n">
+        <v>494</v>
+      </c>
+      <c r="F7" t="n">
+        <v>141</v>
+      </c>
+      <c r="G7" s="10">
+        <f>E7/(E7+F7)</f>
+        <v/>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>majority</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Capital reserve deposit</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>261976</v>
+      </c>
+      <c r="E8" t="n">
+        <v>528</v>
+      </c>
+      <c r="F8" t="n">
+        <v>112</v>
+      </c>
+      <c r="G8" s="10">
+        <f>E8/(E8+F8)</f>
+        <v/>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>majority</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Fire Stations Capital Reserve</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>300000</v>
+      </c>
+      <c r="E9" t="n">
+        <v>365</v>
+      </c>
+      <c r="F9" t="n">
+        <v>268</v>
+      </c>
+      <c r="G9" s="10">
+        <f>E9/(E9+F9)</f>
+        <v/>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>majority</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>PASS (narrow)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>All-Veterans tax credit</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>569</v>
+      </c>
+      <c r="F10" t="n">
+        <v>67</v>
+      </c>
+      <c r="G10" s="10">
+        <f>E10/(E10+F10)</f>
+        <v/>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>majority</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Bond / revolving fund</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>702</v>
+      </c>
+      <c r="F11" t="n">
+        <v>582</v>
+      </c>
+      <c r="G11" s="10">
+        <f>E11/(E11+F11)</f>
+        <v/>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>3/5</t>
+        </is>
+      </c>
+      <c r="I11" s="24" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Capital (3/5)</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>821</v>
+      </c>
+      <c r="F12" t="n">
+        <v>448</v>
+      </c>
+      <c r="G12" s="10">
+        <f>E12/(E12+F12)</f>
+        <v/>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>3/5</t>
+        </is>
+      </c>
+      <c r="I12" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Water / infrastructure</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="E13" t="n">
+        <v>864</v>
+      </c>
+      <c r="F13" t="n">
+        <v>529</v>
+      </c>
+      <c r="G13" s="10">
+        <f>E13/(E13+F13)</f>
+        <v/>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>3/5</t>
+        </is>
+      </c>
+      <c r="I13" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>DWSRF study (100% principal forgiveness)</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E14" t="n">
+        <v>998</v>
+      </c>
+      <c r="F14" t="n">
+        <v>406</v>
+      </c>
+      <c r="G14" s="10">
+        <f>E14/(E14+F14)</f>
+        <v/>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>majority</t>
+        </is>
+      </c>
+      <c r="I14" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Acquire West Swanzey water system</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>822</v>
+      </c>
+      <c r="F15" t="n">
+        <v>553</v>
+      </c>
+      <c r="G15" s="10">
+        <f>E15/(E15+F15)</f>
+        <v/>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>majority</t>
+        </is>
+      </c>
+      <c r="I15" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Ambulance Expendable Trust</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1060</v>
+      </c>
+      <c r="F16" t="n">
+        <v>350</v>
+      </c>
+      <c r="G16" s="10">
+        <f>E16/(E16+F16)</f>
+        <v/>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>majority</t>
+        </is>
+      </c>
+      <c r="I16" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Increase Select Board 3→5</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>740</v>
+      </c>
+      <c r="F17" t="n">
+        <v>653</v>
+      </c>
+      <c r="G17" s="10">
+        <f>E17/(E17+F17)</f>
+        <v/>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>majority</t>
+        </is>
+      </c>
+      <c r="I17" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Second polling location (petition)</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>673</v>
+      </c>
+      <c r="F18" t="n">
+        <v>727</v>
+      </c>
+      <c r="G18" s="10">
+        <f>E18/(E18+F18)</f>
+        <v/>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>majority</t>
+        </is>
+      </c>
+      <c r="I18" s="24" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Public Works Facility ($1.2M)</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="E19" t="n">
+        <v>681</v>
+      </c>
+      <c r="F19" t="n">
+        <v>485</v>
+      </c>
+      <c r="G19" s="10">
+        <f>E19/(E19+F19)</f>
+        <v/>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>3/5</t>
+        </is>
+      </c>
+      <c r="I19" s="24" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Repeal SB2 (return to floor meeting)</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>345</v>
+      </c>
+      <c r="F20" t="n">
+        <v>809</v>
+      </c>
+      <c r="G20" s="10">
+        <f>E20/(E20+F20)</f>
+        <v/>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>majority</t>
+        </is>
+      </c>
+      <c r="I20" s="24" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="C22" s="25" t="inlineStr">
+        <is>
+          <t>Pattern: every bond that needed 3/5 and failed (2024, 2026 facility) still won a MAJORITY. The town will save, not borrow.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Operating-Budget Votes by Town-Meeting Year</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>As-voted margins; support has slid from ~80% to 57%. (2018 &amp; 2020 tallies not machine-readable.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Operating (proposed)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>% YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>5747885</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>5705757</v>
+      </c>
+      <c r="D5" t="n">
+        <v>616</v>
+      </c>
+      <c r="E5" t="n">
+        <v>153</v>
+      </c>
+      <c r="F5" s="10">
+        <f>D5/(D5+E5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>5824380</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>5812387</v>
+      </c>
+      <c r="D6" t="n">
+        <v>436</v>
+      </c>
+      <c r="E6" t="n">
+        <v>131</v>
+      </c>
+      <c r="F6" s="10">
+        <f>D6/(D6+E6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>5888782</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>5821465</v>
+      </c>
+      <c r="D7" t="n">
+        <v>495</v>
+      </c>
+      <c r="E7" t="n">
+        <v>118</v>
+      </c>
+      <c r="F7" s="10">
+        <f>D7/(D7+E7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>6012393</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>5852076</v>
+      </c>
+      <c r="D8" t="n">
+        <v>673</v>
+      </c>
+      <c r="E8" t="n">
+        <v>206</v>
+      </c>
+      <c r="F8" s="10">
+        <f>D8/(D8+E8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>6262426</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>6067144</v>
+      </c>
+      <c r="D9" t="n">
+        <v>670</v>
+      </c>
+      <c r="E9" t="n">
+        <v>311</v>
+      </c>
+      <c r="F9" s="10">
+        <f>D9/(D9+E9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>6210799</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>6222738</v>
+      </c>
+      <c r="D10" t="n">
+        <v>352</v>
+      </c>
+      <c r="E10" t="n">
+        <v>168</v>
+      </c>
+      <c r="F10" s="10">
+        <f>D10/(D10+E10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>6210799</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>6302525</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>6452435</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>6122397</v>
+      </c>
+      <c r="D12" t="n">
+        <v>606</v>
+      </c>
+      <c r="E12" t="n">
+        <v>309</v>
+      </c>
+      <c r="F12" s="10">
+        <f>D12/(D12+E12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>6303000</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>6072735</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>6716500</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>6439109</v>
+      </c>
+      <c r="D14" t="n">
+        <v>637</v>
+      </c>
+      <c r="E14" t="n">
+        <v>460</v>
+      </c>
+      <c r="F14" s="10">
+        <f>D14/(D14+E14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>6902500</v>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>6864706</v>
+      </c>
+      <c r="D15" t="n">
+        <v>751</v>
+      </c>
+      <c r="E15" t="n">
+        <v>262</v>
+      </c>
+      <c r="F15" s="10">
+        <f>D15/(D15+E15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>7425000</v>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>7468834</v>
+      </c>
+      <c r="D16" t="n">
+        <v>388</v>
+      </c>
+      <c r="E16" t="n">
+        <v>236</v>
+      </c>
+      <c r="F16" s="10">
+        <f>D16/(D16+E16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>7961500</v>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>7935699</v>
+      </c>
+      <c r="D17" t="n">
+        <v>738</v>
+      </c>
+      <c r="E17" t="n">
+        <v>530</v>
+      </c>
+      <c r="F17" s="10">
+        <f>D17/(D17+E17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B18" s="9" t="n">
+        <v>8370000</v>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>7935699</v>
+      </c>
+      <c r="D18" t="n">
+        <v>800</v>
+      </c>
+      <c r="E18" t="n">
+        <v>596</v>
+      </c>
+      <c r="F18" s="10">
+        <f>D18/(D18+E18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B19" s="9" t="n">
+        <v>8939036</v>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>8891785</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Select Board Elections &amp; Turnover</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Candidate vote totals where reported; ~ = approximate. Rising volatility compounds administrator churn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Seat</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Votes</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Notable challengers</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3-yr</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Sly Karasinski</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>672</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>strong / uncontested</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>incumbent retained</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>3-yr</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Bill Hutwelker</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>394</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Michael York 216</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>contested</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>seat</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Victoria Reck Ames</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>442</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Brandon Self 418</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>won by 24 — new face</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>3-yr</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>James Tempesta</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>461</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Ward 294, LaBelle 288, Thorne 105</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>crowded field</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>3-yr</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>James Ward</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>545</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Tatro 481, York 414</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>incumbents challenged</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1-yr (new 5th)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Alan Gross</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>678</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Elizabeth Traynor 408</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>first 5th-seat race</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>